<commit_message>
chore(01.2-05): populate Qdrant with 8 CCoP documents
- Ingested 8 CCoP documents via run_ingestion.py
- 87 chunks created (66 unique points in Qdrant)
- Collection: ccop_clauses_hybrid (1024-dim dense + BM25 sparse)
- Verified with 3 retrieval queries: all return relevant results

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ground-truth/phase-2/expert-validation/CCoP_Test_Cases_Expert_Review.xlsx
+++ b/ground-truth/phase-2/expert-validation/CCoP_Test_Cases_Expert_Review.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sagarpratapsingh/dev/sagerstack/studio-ssdlc/ground-truth/phase-2/expert-validation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB4A6CB5-D3A5-B341-9D62-40A34182B2E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50BC2CCB-29BB-5440-A7F4-2FD406122B38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14480" yWindow="-20980" windowWidth="38400" windowHeight="19400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Cases - Expert Review" sheetId="1" r:id="rId1"/>
@@ -3199,8 +3199,8 @@
     <col min="11" max="11" width="80" customWidth="1"/>
     <col min="12" max="12" width="60" customWidth="1"/>
     <col min="13" max="13" width="40" customWidth="1"/>
-    <col min="14" max="14" width="60" customWidth="1"/>
-    <col min="15" max="15" width="40" customWidth="1"/>
+    <col min="14" max="14" width="60" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="40" hidden="1" customWidth="1"/>
     <col min="16" max="16" width="15" style="1" customWidth="1"/>
     <col min="17" max="17" width="60" style="1" customWidth="1"/>
   </cols>

</xml_diff>